<commit_message>
Improve Hanoi validation and confirm positive baselines
</commit_message>
<xml_diff>
--- a/test_corrupt_hanoi.xlsx
+++ b/test_corrupt_hanoi.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -457,6 +457,11 @@
           <t>Human Check</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Targeted Error</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -473,7 +478,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>[2, 3]</t>
+          <t>[2, 3, 4]</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -489,6 +494,11 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>Legal</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>
@@ -497,22 +507,22 @@
         <v>2</v>
       </c>
       <c r="B3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>[3]</t>
+          <t>[2, 3, 4]</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>[2, 1]</t>
+          <t>[1]</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -523,6 +533,11 @@
       <c r="H3" t="inlineStr">
         <is>
           <t>Illegal</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Empty Source Peg</t>
         </is>
       </c>
     </row>
@@ -534,14 +549,14 @@
         <v>1</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>[1, 2, 3]</t>
+          <t>[2, 3, 4]</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -557,6 +572,11 @@
       <c r="H4" t="inlineStr">
         <is>
           <t>Illegal</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Invalid Peg ID</t>
         </is>
       </c>
     </row>
@@ -571,26 +591,31 @@
         <v>1</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>[2]</t>
+          <t>[3, 4]</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[1]</t>
+          <t>[2, 1]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>[3]</t>
+          <t>[99]</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Illegal</t>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Visual Drift</t>
         </is>
       </c>
     </row>
@@ -599,22 +624,22 @@
         <v>5</v>
       </c>
       <c r="B6" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C6" t="n">
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>[2, 3]</t>
+          <t>[3, 4]</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[1]</t>
+          <t>[4, 2, 1]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -625,6 +650,11 @@
       <c r="H6" t="inlineStr">
         <is>
           <t>Illegal</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Size Inversion</t>
         </is>
       </c>
     </row>
@@ -633,22 +663,22 @@
         <v>6</v>
       </c>
       <c r="B7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>[2, 3]</t>
+          <t>[3, 4]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[1]</t>
+          <t>[4, 2, 1]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -659,6 +689,11 @@
       <c r="H7" t="inlineStr">
         <is>
           <t>Illegal</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Ghost Disk</t>
         </is>
       </c>
     </row>
@@ -669,22 +704,20 @@
       <c r="B8" t="n">
         <v>1</v>
       </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>one</t>
-        </is>
+      <c r="C8" t="n">
+        <v>1</v>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>[2, 3]</t>
+          <t>[3, 4]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[1]</t>
+          <t>[4, 2, 1]</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -694,7 +727,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Illegal</t>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Human Discrepancy</t>
         </is>
       </c>
     </row>
@@ -703,7 +741,7 @@
         <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C9" t="n">
         <v>1</v>
@@ -713,22 +751,302 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>[4, 2, 1]</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
           <t>[3]</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" t="n">
+        <v>2</v>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>[2, 1]</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>[4, 3]</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="n">
+        <v>2</v>
+      </c>
+      <c r="C11" t="n">
+        <v>2</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[2, 4]</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
         <is>
           <t>[1]</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>[99]</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>[4, 3]</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>Legal</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[2, 4]</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>[4, 3]</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Illegal</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Identical Pegs</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>one</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[2, 4]</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>[4, 3]</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Illegal</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Malformed Data</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>[4]</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>[2, 1]</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>[4, 3]</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>[2, 1]</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>[4, 4, 3]</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="n">
+        <v>1</v>
+      </c>
+      <c r="C16" t="n">
+        <v>2</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>[1]</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>[2, 4, 4, 3]</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Legal</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>None</t>
         </is>
       </c>
     </row>

</xml_diff>